<commit_message>
fix(privacy): namuna Excel fayllaridan haqiqiy korxona va shaxs ma'lumotlarini olib tashlash
Fayllar saytdan ommaviy yuklab olinadi, lekin ichida haqiqiy hisobot qolgan edi.

Olib tashlandi (ikkala faylda):
- korxona nomi -> "NAMUNA KORXONA"
- hudud, manzil -> "—"
- rahbar va bosh hisobchi ismlari -> "—"
- OKPO, STIR (INN), SOATO raqamlari -> bo'sh katak
- hujjat metama'lumoti (dc:creator, cp:lastModifiedBy, Company) -> "Digital CFO"

Moliyaviy raqamlar o'zgarmadi: balans varaqlaridagi barcha kataklar joyida
(sheet2/sheet4 -- 97 va 161 ta raqamli katak), namuna sifatida ishlatish mumkin.

Tekshirildi: zip butunligi OK, arxiv bo'ylab qidiruvda qoldiq yo'q.
Namuna_Moliyaviy_Hisobot.pdf allaqachon toza edi (Korxona/STIR maydonlari bo'sh),
tegilmadi.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/Shakl_1_Balans_namuna.xlsx
+++ b/client/public/Shakl_1_Balans_namuna.xlsx
@@ -1165,7 +1165,7 @@
     <t>по ОКЕД</t>
   </si>
   <si>
-    <t>"O`ZAGROLIZING" AKSIYADORLIK JAMIYATI</t>
+    <t>NAMUNA KORXONA</t>
   </si>
   <si>
     <t>НЕТ ДАННЫХ В СПРАВОЧНИКЕ</t>
@@ -1180,10 +1180,10 @@
     <t>06244</t>
   </si>
   <si>
-    <t>ТОШКЕНТ ШАҲАР ЯККАСАРОЙ тумани</t>
-  </si>
-  <si>
-    <t>BOBUR KO`CHASI 42 А</t>
+    <t>—</t>
+  </si>
+  <si>
+    <t>—</t>
   </si>
   <si>
     <t>17.04.2026</t>
@@ -1192,10 +1192,10 @@
     <t>27.04.2026</t>
   </si>
   <si>
-    <t>NASIRDINOV AZIMJON SHOMAXMUDOVICH</t>
-  </si>
-  <si>
-    <t>QODIROVA SHAHNOZA SHUKURJON QIZI</t>
+    <t>—</t>
+  </si>
+  <si>
+    <t>—</t>
   </si>
   <si>
     <t>I квартал</t>
@@ -2099,9 +2099,7 @@
       <c r="H7" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="I7" s="38">
-        <v>17489494</v>
-      </c>
+      <c r="I7" s="38"/>
     </row>
     <row r="8" spans="1:9" ht="3.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="53"/>
@@ -2233,9 +2231,7 @@
       <c r="H17" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="I17" s="39">
-        <v>203071206</v>
-      </c>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="2:9" ht="3.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="53"/>
@@ -2261,9 +2257,7 @@
       <c r="H19" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="I19" s="39">
-        <v>1726287</v>
-      </c>
+      <c r="I19" s="39"/>
     </row>
     <row r="20" spans="2:9" ht="3.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="53"/>

</xml_diff>